<commit_message>
added data to cherokee
</commit_message>
<xml_diff>
--- a/DawesRollsViewer/Dawes Rolls One Document/Cherokee/Cherokee By InterMarriage.xlsx
+++ b/DawesRollsViewer/Dawes Rolls One Document/Cherokee/Cherokee By InterMarriage.xlsx
@@ -390,7 +390,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O289"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -440,6 +440,1733 @@
         <v>14</v>
       </c>
     </row>
+    <row r="2" spans="1:15">
+      <c r="A2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3">
+        <f>A2+1</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4">
+        <f t="shared" ref="A4:A67" si="0">A3+1</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="A5">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
+      <c r="A13">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
+      <c r="A14">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
+      <c r="A15">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
+      <c r="A16">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56">
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57">
+        <f t="shared" si="0"/>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58">
+        <f t="shared" si="0"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62">
+        <f t="shared" si="0"/>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63">
+        <f t="shared" si="0"/>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64">
+        <f t="shared" si="0"/>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67">
+        <f t="shared" si="0"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68">
+        <f t="shared" ref="A68:A131" si="1">A67+1</f>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69">
+        <f t="shared" si="1"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70">
+        <f t="shared" si="1"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71">
+        <f t="shared" si="1"/>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72">
+        <f t="shared" si="1"/>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73">
+        <f t="shared" si="1"/>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74">
+        <f t="shared" si="1"/>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75">
+        <f t="shared" si="1"/>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77">
+        <f t="shared" si="1"/>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78">
+        <f t="shared" si="1"/>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79">
+        <f t="shared" si="1"/>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80">
+        <f t="shared" si="1"/>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82">
+        <f t="shared" si="1"/>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83">
+        <f t="shared" si="1"/>
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84">
+        <f t="shared" si="1"/>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85">
+        <f t="shared" si="1"/>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86">
+        <f t="shared" si="1"/>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1">
+      <c r="A87">
+        <f t="shared" si="1"/>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88">
+        <f t="shared" si="1"/>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1">
+      <c r="A89">
+        <f t="shared" si="1"/>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90">
+        <f t="shared" si="1"/>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91">
+        <f t="shared" si="1"/>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92">
+        <f t="shared" si="1"/>
+        <v>91</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1">
+      <c r="A93">
+        <f t="shared" si="1"/>
+        <v>92</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94">
+        <f t="shared" si="1"/>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95">
+        <f t="shared" si="1"/>
+        <v>94</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96">
+        <f t="shared" si="1"/>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97">
+        <f t="shared" si="1"/>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98">
+        <f t="shared" si="1"/>
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99">
+        <f t="shared" si="1"/>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100">
+        <f t="shared" si="1"/>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102">
+        <f t="shared" si="1"/>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103">
+        <f t="shared" si="1"/>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104">
+        <f t="shared" si="1"/>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105">
+        <f t="shared" si="1"/>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106">
+        <f t="shared" si="1"/>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107">
+        <f t="shared" si="1"/>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108">
+        <f t="shared" si="1"/>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1">
+      <c r="A109">
+        <f t="shared" si="1"/>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110">
+        <f t="shared" si="1"/>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1">
+      <c r="A111">
+        <f t="shared" si="1"/>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112">
+        <f t="shared" si="1"/>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113">
+        <f t="shared" si="1"/>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114">
+        <f t="shared" si="1"/>
+        <v>113</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115">
+        <f t="shared" si="1"/>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1">
+      <c r="A116">
+        <f t="shared" si="1"/>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117">
+        <f t="shared" si="1"/>
+        <v>116</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1">
+      <c r="A118">
+        <f t="shared" si="1"/>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1">
+      <c r="A119">
+        <f t="shared" si="1"/>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1">
+      <c r="A120">
+        <f t="shared" si="1"/>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1">
+      <c r="A121">
+        <f t="shared" si="1"/>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1">
+      <c r="A122">
+        <f t="shared" si="1"/>
+        <v>121</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1">
+      <c r="A123">
+        <f t="shared" si="1"/>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1">
+      <c r="A124">
+        <f t="shared" si="1"/>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1">
+      <c r="A125">
+        <f t="shared" si="1"/>
+        <v>124</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1">
+      <c r="A126">
+        <f t="shared" si="1"/>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1">
+      <c r="A127">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1">
+      <c r="A128">
+        <f t="shared" si="1"/>
+        <v>127</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1">
+      <c r="A129">
+        <f t="shared" si="1"/>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1">
+      <c r="A130">
+        <f t="shared" si="1"/>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1">
+      <c r="A131">
+        <f t="shared" si="1"/>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1">
+      <c r="A132">
+        <f t="shared" ref="A132:A195" si="2">A131+1</f>
+        <v>131</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1">
+      <c r="A133">
+        <f t="shared" si="2"/>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1">
+      <c r="A134">
+        <f t="shared" si="2"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1">
+      <c r="A135">
+        <f t="shared" si="2"/>
+        <v>134</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1">
+      <c r="A136">
+        <f t="shared" si="2"/>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1">
+      <c r="A137">
+        <f t="shared" si="2"/>
+        <v>136</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1">
+      <c r="A138">
+        <f t="shared" si="2"/>
+        <v>137</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1">
+      <c r="A139">
+        <f t="shared" si="2"/>
+        <v>138</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1">
+      <c r="A140">
+        <f t="shared" si="2"/>
+        <v>139</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1">
+      <c r="A141">
+        <f t="shared" si="2"/>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1">
+      <c r="A142">
+        <f t="shared" si="2"/>
+        <v>141</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1">
+      <c r="A143">
+        <f t="shared" si="2"/>
+        <v>142</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1">
+      <c r="A144">
+        <f t="shared" si="2"/>
+        <v>143</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1">
+      <c r="A145">
+        <f t="shared" si="2"/>
+        <v>144</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1">
+      <c r="A146">
+        <f t="shared" si="2"/>
+        <v>145</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1">
+      <c r="A147">
+        <f t="shared" si="2"/>
+        <v>146</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1">
+      <c r="A148">
+        <f t="shared" si="2"/>
+        <v>147</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1">
+      <c r="A149">
+        <f t="shared" si="2"/>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1">
+      <c r="A150">
+        <f t="shared" si="2"/>
+        <v>149</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1">
+      <c r="A151">
+        <f t="shared" si="2"/>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1">
+      <c r="A152">
+        <f t="shared" si="2"/>
+        <v>151</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1">
+      <c r="A153">
+        <f t="shared" si="2"/>
+        <v>152</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1">
+      <c r="A154">
+        <f t="shared" si="2"/>
+        <v>153</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1">
+      <c r="A155">
+        <f t="shared" si="2"/>
+        <v>154</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1">
+      <c r="A156">
+        <f t="shared" si="2"/>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1">
+      <c r="A157">
+        <f t="shared" si="2"/>
+        <v>156</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1">
+      <c r="A158">
+        <f t="shared" si="2"/>
+        <v>157</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1">
+      <c r="A159">
+        <f t="shared" si="2"/>
+        <v>158</v>
+      </c>
+    </row>
+    <row r="160" spans="1:1">
+      <c r="A160">
+        <f t="shared" si="2"/>
+        <v>159</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1">
+      <c r="A161">
+        <f t="shared" si="2"/>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1">
+      <c r="A162">
+        <f t="shared" si="2"/>
+        <v>161</v>
+      </c>
+    </row>
+    <row r="163" spans="1:1">
+      <c r="A163">
+        <f t="shared" si="2"/>
+        <v>162</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1">
+      <c r="A164">
+        <f t="shared" si="2"/>
+        <v>163</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1">
+      <c r="A165">
+        <f t="shared" si="2"/>
+        <v>164</v>
+      </c>
+    </row>
+    <row r="166" spans="1:1">
+      <c r="A166">
+        <f t="shared" si="2"/>
+        <v>165</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1">
+      <c r="A167">
+        <f t="shared" si="2"/>
+        <v>166</v>
+      </c>
+    </row>
+    <row r="168" spans="1:1">
+      <c r="A168">
+        <f t="shared" si="2"/>
+        <v>167</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1">
+      <c r="A169">
+        <f t="shared" si="2"/>
+        <v>168</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1">
+      <c r="A170">
+        <f t="shared" si="2"/>
+        <v>169</v>
+      </c>
+    </row>
+    <row r="171" spans="1:1">
+      <c r="A171">
+        <f t="shared" si="2"/>
+        <v>170</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1">
+      <c r="A172">
+        <f t="shared" si="2"/>
+        <v>171</v>
+      </c>
+    </row>
+    <row r="173" spans="1:1">
+      <c r="A173">
+        <f t="shared" si="2"/>
+        <v>172</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1">
+      <c r="A174">
+        <f t="shared" si="2"/>
+        <v>173</v>
+      </c>
+    </row>
+    <row r="175" spans="1:1">
+      <c r="A175">
+        <f t="shared" si="2"/>
+        <v>174</v>
+      </c>
+    </row>
+    <row r="176" spans="1:1">
+      <c r="A176">
+        <f t="shared" si="2"/>
+        <v>175</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1">
+      <c r="A177">
+        <f t="shared" si="2"/>
+        <v>176</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1">
+      <c r="A178">
+        <f t="shared" si="2"/>
+        <v>177</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1">
+      <c r="A179">
+        <f t="shared" si="2"/>
+        <v>178</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1">
+      <c r="A180">
+        <f t="shared" si="2"/>
+        <v>179</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1">
+      <c r="A181">
+        <f t="shared" si="2"/>
+        <v>180</v>
+      </c>
+    </row>
+    <row r="182" spans="1:1">
+      <c r="A182">
+        <f t="shared" si="2"/>
+        <v>181</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1">
+      <c r="A183">
+        <f t="shared" si="2"/>
+        <v>182</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1">
+      <c r="A184">
+        <f t="shared" si="2"/>
+        <v>183</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1">
+      <c r="A185">
+        <f t="shared" si="2"/>
+        <v>184</v>
+      </c>
+    </row>
+    <row r="186" spans="1:1">
+      <c r="A186">
+        <f t="shared" si="2"/>
+        <v>185</v>
+      </c>
+    </row>
+    <row r="187" spans="1:1">
+      <c r="A187">
+        <f t="shared" si="2"/>
+        <v>186</v>
+      </c>
+    </row>
+    <row r="188" spans="1:1">
+      <c r="A188">
+        <f t="shared" si="2"/>
+        <v>187</v>
+      </c>
+    </row>
+    <row r="189" spans="1:1">
+      <c r="A189">
+        <f t="shared" si="2"/>
+        <v>188</v>
+      </c>
+    </row>
+    <row r="190" spans="1:1">
+      <c r="A190">
+        <f t="shared" si="2"/>
+        <v>189</v>
+      </c>
+    </row>
+    <row r="191" spans="1:1">
+      <c r="A191">
+        <f t="shared" si="2"/>
+        <v>190</v>
+      </c>
+    </row>
+    <row r="192" spans="1:1">
+      <c r="A192">
+        <f t="shared" si="2"/>
+        <v>191</v>
+      </c>
+    </row>
+    <row r="193" spans="1:1">
+      <c r="A193">
+        <f t="shared" si="2"/>
+        <v>192</v>
+      </c>
+    </row>
+    <row r="194" spans="1:1">
+      <c r="A194">
+        <f t="shared" si="2"/>
+        <v>193</v>
+      </c>
+    </row>
+    <row r="195" spans="1:1">
+      <c r="A195">
+        <f t="shared" si="2"/>
+        <v>194</v>
+      </c>
+    </row>
+    <row r="196" spans="1:1">
+      <c r="A196">
+        <f t="shared" ref="A196:A259" si="3">A195+1</f>
+        <v>195</v>
+      </c>
+    </row>
+    <row r="197" spans="1:1">
+      <c r="A197">
+        <f t="shared" si="3"/>
+        <v>196</v>
+      </c>
+    </row>
+    <row r="198" spans="1:1">
+      <c r="A198">
+        <f t="shared" si="3"/>
+        <v>197</v>
+      </c>
+    </row>
+    <row r="199" spans="1:1">
+      <c r="A199">
+        <f t="shared" si="3"/>
+        <v>198</v>
+      </c>
+    </row>
+    <row r="200" spans="1:1">
+      <c r="A200">
+        <f t="shared" si="3"/>
+        <v>199</v>
+      </c>
+    </row>
+    <row r="201" spans="1:1">
+      <c r="A201">
+        <f t="shared" si="3"/>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="202" spans="1:1">
+      <c r="A202">
+        <f t="shared" si="3"/>
+        <v>201</v>
+      </c>
+    </row>
+    <row r="203" spans="1:1">
+      <c r="A203">
+        <f t="shared" si="3"/>
+        <v>202</v>
+      </c>
+    </row>
+    <row r="204" spans="1:1">
+      <c r="A204">
+        <f t="shared" si="3"/>
+        <v>203</v>
+      </c>
+    </row>
+    <row r="205" spans="1:1">
+      <c r="A205">
+        <f t="shared" si="3"/>
+        <v>204</v>
+      </c>
+    </row>
+    <row r="206" spans="1:1">
+      <c r="A206">
+        <f t="shared" si="3"/>
+        <v>205</v>
+      </c>
+    </row>
+    <row r="207" spans="1:1">
+      <c r="A207">
+        <f t="shared" si="3"/>
+        <v>206</v>
+      </c>
+    </row>
+    <row r="208" spans="1:1">
+      <c r="A208">
+        <f t="shared" si="3"/>
+        <v>207</v>
+      </c>
+    </row>
+    <row r="209" spans="1:1">
+      <c r="A209">
+        <f t="shared" si="3"/>
+        <v>208</v>
+      </c>
+    </row>
+    <row r="210" spans="1:1">
+      <c r="A210">
+        <f t="shared" si="3"/>
+        <v>209</v>
+      </c>
+    </row>
+    <row r="211" spans="1:1">
+      <c r="A211">
+        <f t="shared" si="3"/>
+        <v>210</v>
+      </c>
+    </row>
+    <row r="212" spans="1:1">
+      <c r="A212">
+        <f t="shared" si="3"/>
+        <v>211</v>
+      </c>
+    </row>
+    <row r="213" spans="1:1">
+      <c r="A213">
+        <f t="shared" si="3"/>
+        <v>212</v>
+      </c>
+    </row>
+    <row r="214" spans="1:1">
+      <c r="A214">
+        <f t="shared" si="3"/>
+        <v>213</v>
+      </c>
+    </row>
+    <row r="215" spans="1:1">
+      <c r="A215">
+        <f t="shared" si="3"/>
+        <v>214</v>
+      </c>
+    </row>
+    <row r="216" spans="1:1">
+      <c r="A216">
+        <f t="shared" si="3"/>
+        <v>215</v>
+      </c>
+    </row>
+    <row r="217" spans="1:1">
+      <c r="A217">
+        <f t="shared" si="3"/>
+        <v>216</v>
+      </c>
+    </row>
+    <row r="218" spans="1:1">
+      <c r="A218">
+        <f t="shared" si="3"/>
+        <v>217</v>
+      </c>
+    </row>
+    <row r="219" spans="1:1">
+      <c r="A219">
+        <f t="shared" si="3"/>
+        <v>218</v>
+      </c>
+    </row>
+    <row r="220" spans="1:1">
+      <c r="A220">
+        <f t="shared" si="3"/>
+        <v>219</v>
+      </c>
+    </row>
+    <row r="221" spans="1:1">
+      <c r="A221">
+        <f t="shared" si="3"/>
+        <v>220</v>
+      </c>
+    </row>
+    <row r="222" spans="1:1">
+      <c r="A222">
+        <f t="shared" si="3"/>
+        <v>221</v>
+      </c>
+    </row>
+    <row r="223" spans="1:1">
+      <c r="A223">
+        <f t="shared" si="3"/>
+        <v>222</v>
+      </c>
+    </row>
+    <row r="224" spans="1:1">
+      <c r="A224">
+        <f t="shared" si="3"/>
+        <v>223</v>
+      </c>
+    </row>
+    <row r="225" spans="1:1">
+      <c r="A225">
+        <f t="shared" si="3"/>
+        <v>224</v>
+      </c>
+    </row>
+    <row r="226" spans="1:1">
+      <c r="A226">
+        <f t="shared" si="3"/>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="227" spans="1:1">
+      <c r="A227">
+        <f t="shared" si="3"/>
+        <v>226</v>
+      </c>
+    </row>
+    <row r="228" spans="1:1">
+      <c r="A228">
+        <f t="shared" si="3"/>
+        <v>227</v>
+      </c>
+    </row>
+    <row r="229" spans="1:1">
+      <c r="A229">
+        <f t="shared" si="3"/>
+        <v>228</v>
+      </c>
+    </row>
+    <row r="230" spans="1:1">
+      <c r="A230">
+        <f t="shared" si="3"/>
+        <v>229</v>
+      </c>
+    </row>
+    <row r="231" spans="1:1">
+      <c r="A231">
+        <f t="shared" si="3"/>
+        <v>230</v>
+      </c>
+    </row>
+    <row r="232" spans="1:1">
+      <c r="A232">
+        <f t="shared" si="3"/>
+        <v>231</v>
+      </c>
+    </row>
+    <row r="233" spans="1:1">
+      <c r="A233">
+        <f t="shared" si="3"/>
+        <v>232</v>
+      </c>
+    </row>
+    <row r="234" spans="1:1">
+      <c r="A234">
+        <f t="shared" si="3"/>
+        <v>233</v>
+      </c>
+    </row>
+    <row r="235" spans="1:1">
+      <c r="A235">
+        <f t="shared" si="3"/>
+        <v>234</v>
+      </c>
+    </row>
+    <row r="236" spans="1:1">
+      <c r="A236">
+        <f t="shared" si="3"/>
+        <v>235</v>
+      </c>
+    </row>
+    <row r="237" spans="1:1">
+      <c r="A237">
+        <f t="shared" si="3"/>
+        <v>236</v>
+      </c>
+    </row>
+    <row r="238" spans="1:1">
+      <c r="A238">
+        <f t="shared" si="3"/>
+        <v>237</v>
+      </c>
+    </row>
+    <row r="239" spans="1:1">
+      <c r="A239">
+        <f t="shared" si="3"/>
+        <v>238</v>
+      </c>
+    </row>
+    <row r="240" spans="1:1">
+      <c r="A240">
+        <f t="shared" si="3"/>
+        <v>239</v>
+      </c>
+    </row>
+    <row r="241" spans="1:1">
+      <c r="A241">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="242" spans="1:1">
+      <c r="A242">
+        <f t="shared" si="3"/>
+        <v>241</v>
+      </c>
+    </row>
+    <row r="243" spans="1:1">
+      <c r="A243">
+        <f t="shared" si="3"/>
+        <v>242</v>
+      </c>
+    </row>
+    <row r="244" spans="1:1">
+      <c r="A244">
+        <f t="shared" si="3"/>
+        <v>243</v>
+      </c>
+    </row>
+    <row r="245" spans="1:1">
+      <c r="A245">
+        <f t="shared" si="3"/>
+        <v>244</v>
+      </c>
+    </row>
+    <row r="246" spans="1:1">
+      <c r="A246">
+        <f t="shared" si="3"/>
+        <v>245</v>
+      </c>
+    </row>
+    <row r="247" spans="1:1">
+      <c r="A247">
+        <f t="shared" si="3"/>
+        <v>246</v>
+      </c>
+    </row>
+    <row r="248" spans="1:1">
+      <c r="A248">
+        <f t="shared" si="3"/>
+        <v>247</v>
+      </c>
+    </row>
+    <row r="249" spans="1:1">
+      <c r="A249">
+        <f t="shared" si="3"/>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="250" spans="1:1">
+      <c r="A250">
+        <f t="shared" si="3"/>
+        <v>249</v>
+      </c>
+    </row>
+    <row r="251" spans="1:1">
+      <c r="A251">
+        <f t="shared" si="3"/>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="252" spans="1:1">
+      <c r="A252">
+        <f t="shared" si="3"/>
+        <v>251</v>
+      </c>
+    </row>
+    <row r="253" spans="1:1">
+      <c r="A253">
+        <f t="shared" si="3"/>
+        <v>252</v>
+      </c>
+    </row>
+    <row r="254" spans="1:1">
+      <c r="A254">
+        <f t="shared" si="3"/>
+        <v>253</v>
+      </c>
+    </row>
+    <row r="255" spans="1:1">
+      <c r="A255">
+        <f t="shared" si="3"/>
+        <v>254</v>
+      </c>
+    </row>
+    <row r="256" spans="1:1">
+      <c r="A256">
+        <f t="shared" si="3"/>
+        <v>255</v>
+      </c>
+    </row>
+    <row r="257" spans="1:1">
+      <c r="A257">
+        <f t="shared" si="3"/>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="258" spans="1:1">
+      <c r="A258">
+        <f t="shared" si="3"/>
+        <v>257</v>
+      </c>
+    </row>
+    <row r="259" spans="1:1">
+      <c r="A259">
+        <f t="shared" si="3"/>
+        <v>258</v>
+      </c>
+    </row>
+    <row r="260" spans="1:1">
+      <c r="A260">
+        <f t="shared" ref="A260:A289" si="4">A259+1</f>
+        <v>259</v>
+      </c>
+    </row>
+    <row r="261" spans="1:1">
+      <c r="A261">
+        <f t="shared" si="4"/>
+        <v>260</v>
+      </c>
+    </row>
+    <row r="262" spans="1:1">
+      <c r="A262">
+        <f t="shared" si="4"/>
+        <v>261</v>
+      </c>
+    </row>
+    <row r="263" spans="1:1">
+      <c r="A263">
+        <f t="shared" si="4"/>
+        <v>262</v>
+      </c>
+    </row>
+    <row r="264" spans="1:1">
+      <c r="A264">
+        <f t="shared" si="4"/>
+        <v>263</v>
+      </c>
+    </row>
+    <row r="265" spans="1:1">
+      <c r="A265">
+        <f t="shared" si="4"/>
+        <v>264</v>
+      </c>
+    </row>
+    <row r="266" spans="1:1">
+      <c r="A266">
+        <f t="shared" si="4"/>
+        <v>265</v>
+      </c>
+    </row>
+    <row r="267" spans="1:1">
+      <c r="A267">
+        <f t="shared" si="4"/>
+        <v>266</v>
+      </c>
+    </row>
+    <row r="268" spans="1:1">
+      <c r="A268">
+        <f t="shared" si="4"/>
+        <v>267</v>
+      </c>
+    </row>
+    <row r="269" spans="1:1">
+      <c r="A269">
+        <f t="shared" si="4"/>
+        <v>268</v>
+      </c>
+    </row>
+    <row r="270" spans="1:1">
+      <c r="A270">
+        <f t="shared" si="4"/>
+        <v>269</v>
+      </c>
+    </row>
+    <row r="271" spans="1:1">
+      <c r="A271">
+        <f t="shared" si="4"/>
+        <v>270</v>
+      </c>
+    </row>
+    <row r="272" spans="1:1">
+      <c r="A272">
+        <f t="shared" si="4"/>
+        <v>271</v>
+      </c>
+    </row>
+    <row r="273" spans="1:1">
+      <c r="A273">
+        <f t="shared" si="4"/>
+        <v>272</v>
+      </c>
+    </row>
+    <row r="274" spans="1:1">
+      <c r="A274">
+        <f t="shared" si="4"/>
+        <v>273</v>
+      </c>
+    </row>
+    <row r="275" spans="1:1">
+      <c r="A275">
+        <f t="shared" si="4"/>
+        <v>274</v>
+      </c>
+    </row>
+    <row r="276" spans="1:1">
+      <c r="A276">
+        <f t="shared" si="4"/>
+        <v>275</v>
+      </c>
+    </row>
+    <row r="277" spans="1:1">
+      <c r="A277">
+        <f t="shared" si="4"/>
+        <v>276</v>
+      </c>
+    </row>
+    <row r="278" spans="1:1">
+      <c r="A278">
+        <f t="shared" si="4"/>
+        <v>277</v>
+      </c>
+    </row>
+    <row r="279" spans="1:1">
+      <c r="A279">
+        <f t="shared" si="4"/>
+        <v>278</v>
+      </c>
+    </row>
+    <row r="280" spans="1:1">
+      <c r="A280">
+        <f t="shared" si="4"/>
+        <v>279</v>
+      </c>
+    </row>
+    <row r="281" spans="1:1">
+      <c r="A281">
+        <f t="shared" si="4"/>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="282" spans="1:1">
+      <c r="A282">
+        <f t="shared" si="4"/>
+        <v>281</v>
+      </c>
+    </row>
+    <row r="283" spans="1:1">
+      <c r="A283">
+        <f t="shared" si="4"/>
+        <v>282</v>
+      </c>
+    </row>
+    <row r="284" spans="1:1">
+      <c r="A284">
+        <f t="shared" si="4"/>
+        <v>283</v>
+      </c>
+    </row>
+    <row r="285" spans="1:1">
+      <c r="A285">
+        <f t="shared" si="4"/>
+        <v>284</v>
+      </c>
+    </row>
+    <row r="286" spans="1:1">
+      <c r="A286">
+        <f t="shared" si="4"/>
+        <v>285</v>
+      </c>
+    </row>
+    <row r="287" spans="1:1">
+      <c r="A287">
+        <f t="shared" si="4"/>
+        <v>286</v>
+      </c>
+    </row>
+    <row r="288" spans="1:1">
+      <c r="A288">
+        <f t="shared" si="4"/>
+        <v>287</v>
+      </c>
+    </row>
+    <row r="289" spans="1:1">
+      <c r="A289">
+        <f t="shared" si="4"/>
+        <v>288</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added data to dawes rolls
</commit_message>
<xml_diff>
--- a/DawesRollsViewer/Dawes Rolls One Document/Cherokee/Cherokee By InterMarriage.xlsx
+++ b/DawesRollsViewer/Dawes Rolls One Document/Cherokee/Cherokee By InterMarriage.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="22">
   <si>
     <t>ID</t>
   </si>
@@ -74,6 +74,12 @@
   </si>
   <si>
     <t>Dawes Rolls Full Document - Cherokee By Blood - Page 472</t>
+  </si>
+  <si>
+    <t>Image Name</t>
+  </si>
+  <si>
+    <t>Image Binary</t>
   </si>
 </sst>
 </file>
@@ -405,14 +411,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O289"/>
+  <dimension ref="A1:Q289"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="13.140625" customWidth="1"/>
     <col min="14" max="14" width="57.140625" customWidth="1"/>
+    <col min="16" max="16" width="13.42578125" customWidth="1"/>
+    <col min="17" max="17" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -458,8 +466,14 @@
       <c r="O1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:15">
+      <c r="P1" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2">
         <v>1</v>
       </c>
@@ -476,7 +490,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:17">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -496,7 +510,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:17">
       <c r="A4">
         <f t="shared" ref="A4:A67" si="0">A3+1</f>
         <v>3</v>
@@ -516,7 +530,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:17">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -536,7 +550,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:17">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -556,7 +570,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:17">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -576,7 +590,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:17">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -596,7 +610,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:17">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -616,7 +630,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:17">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -636,7 +650,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:17">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -656,7 +670,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:17">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -676,7 +690,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:17">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -696,7 +710,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:17">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -716,7 +730,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:17">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -736,7 +750,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:17">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>15</v>

</xml_diff>

<commit_message>
added data for cherokee intermarriage
</commit_message>
<xml_diff>
--- a/DawesRollsViewer/Dawes Rolls One Document/Cherokee/Cherokee By InterMarriage.xlsx
+++ b/DawesRollsViewer/Dawes Rolls One Document/Cherokee/Cherokee By InterMarriage.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="24">
   <si>
     <t>ID</t>
   </si>
@@ -80,6 +80,12 @@
   </si>
   <si>
     <t>Image Binary</t>
+  </si>
+  <si>
+    <t>Stricken From Roll</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -5218,8 +5224,35 @@
         <f t="shared" si="12"/>
         <v>472</v>
       </c>
+      <c r="D239" t="s">
+        <v>22</v>
+      </c>
+      <c r="E239" t="s">
+        <v>23</v>
+      </c>
+      <c r="F239" t="s">
+        <v>23</v>
+      </c>
+      <c r="G239" t="s">
+        <v>23</v>
+      </c>
+      <c r="H239">
+        <v>-1</v>
+      </c>
+      <c r="I239" t="s">
+        <v>23</v>
+      </c>
+      <c r="J239" t="s">
+        <v>23</v>
+      </c>
+      <c r="K239" t="s">
+        <v>23</v>
+      </c>
       <c r="L239" t="s">
-        <v>15</v>
+        <v>23</v>
+      </c>
+      <c r="M239" t="s">
+        <v>23</v>
       </c>
       <c r="N239" t="str">
         <f t="shared" si="13"/>
@@ -5238,8 +5271,35 @@
         <f t="shared" si="12"/>
         <v>472</v>
       </c>
+      <c r="D240" t="s">
+        <v>22</v>
+      </c>
+      <c r="E240" t="s">
+        <v>23</v>
+      </c>
+      <c r="F240" t="s">
+        <v>23</v>
+      </c>
+      <c r="G240" t="s">
+        <v>23</v>
+      </c>
+      <c r="H240">
+        <v>0</v>
+      </c>
+      <c r="I240" t="s">
+        <v>23</v>
+      </c>
+      <c r="J240" t="s">
+        <v>23</v>
+      </c>
+      <c r="K240" t="s">
+        <v>23</v>
+      </c>
       <c r="L240" t="s">
-        <v>15</v>
+        <v>23</v>
+      </c>
+      <c r="M240" t="s">
+        <v>23</v>
       </c>
       <c r="N240" t="str">
         <f t="shared" si="13"/>

</xml_diff>

<commit_message>
added more changes to the app
</commit_message>
<xml_diff>
--- a/DawesRollsViewer/Dawes Rolls One Document/Cherokee/Cherokee By InterMarriage.xlsx
+++ b/DawesRollsViewer/Dawes Rolls One Document/Cherokee/Cherokee By InterMarriage.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="25">
   <si>
     <t>ID</t>
   </si>
@@ -76,16 +76,19 @@
     <t>Dawes Rolls Full Document - Cherokee By Blood - Page 472</t>
   </si>
   <si>
-    <t>Image Name</t>
-  </si>
-  <si>
-    <t>Image Binary</t>
-  </si>
-  <si>
     <t>Stricken From Roll</t>
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>ImageName</t>
+  </si>
+  <si>
+    <t>ImageBinary</t>
+  </si>
+  <si>
+    <t>TribeRelationship</t>
   </si>
 </sst>
 </file>
@@ -417,16 +420,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q289"/>
+  <dimension ref="A1:R289"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="13.140625" customWidth="1"/>
     <col min="14" max="14" width="57.140625" customWidth="1"/>
     <col min="16" max="16" width="13.42578125" customWidth="1"/>
     <col min="17" max="17" width="14" customWidth="1"/>
+    <col min="18" max="18" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:18">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -473,13 +477,16 @@
         <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="Q1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17">
+        <v>23</v>
+      </c>
+      <c r="R1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18">
       <c r="A2">
         <v>1</v>
       </c>
@@ -496,7 +503,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:18">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -516,7 +523,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:18">
       <c r="A4">
         <f t="shared" ref="A4:A67" si="0">A3+1</f>
         <v>3</v>
@@ -536,7 +543,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:18">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -556,7 +563,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:18">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -576,7 +583,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:18">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -596,7 +603,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:18">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -616,7 +623,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:18">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -636,7 +643,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:18">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -656,7 +663,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:18">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -676,7 +683,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:18">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -696,7 +703,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:18">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -716,7 +723,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:18">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -736,7 +743,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:18">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -756,7 +763,7 @@
         <v>Dawes Rolls Full Document - Cherokee By Blood - Page 470</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:18">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -5225,34 +5232,34 @@
         <v>472</v>
       </c>
       <c r="D239" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E239" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F239" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G239" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H239">
         <v>-1</v>
       </c>
       <c r="I239" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J239" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K239" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="L239" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M239" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="N239" t="str">
         <f t="shared" si="13"/>
@@ -5272,34 +5279,34 @@
         <v>472</v>
       </c>
       <c r="D240" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E240" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F240" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G240" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H240">
         <v>0</v>
       </c>
       <c r="I240" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J240" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K240" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="L240" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M240" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="N240" t="str">
         <f t="shared" si="13"/>

</xml_diff>